<commit_message>
Custom Editor List sorted
</commit_message>
<xml_diff>
--- a/Bug Tracker.xlsx
+++ b/Bug Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Uni Work\Year 3\FMP\ProcGenTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97AB2AD5-5A9E-410E-9CC8-DEAB2AEB446A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB76808-A26A-4BE2-9F81-123446888FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{96347398-2AC3-4EB9-A82F-8E2B65190871}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>Bug Tracker</t>
   </si>
@@ -177,6 +177,24 @@
   </si>
   <si>
     <t>Set tiles to hollow (transparent) instead of null</t>
+  </si>
+  <si>
+    <t>List not displaying properly</t>
+  </si>
+  <si>
+    <t>CustomEditorWindow.cs</t>
+  </si>
+  <si>
+    <t>Changed EditorGUI to EditorGUILayout</t>
+  </si>
+  <si>
+    <t>Wrong class call</t>
+  </si>
+  <si>
+    <t>Plus and minus missing</t>
+  </si>
+  <si>
+    <t>Tiles changed from null to hollow</t>
   </si>
 </sst>
 </file>
@@ -894,7 +912,9 @@
       <c r="K12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L12" s="1"/>
+      <c r="L12" s="1" t="s">
+        <v>52</v>
+      </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
@@ -934,17 +954,27 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="1"/>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="E14" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="H14" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
@@ -954,16 +984,22 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="1"/>
+      <c r="B15" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="H15" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>

</xml_diff>

<commit_message>
Added readme and tested packaging
</commit_message>
<xml_diff>
--- a/Bug Tracker.xlsx
+++ b/Bug Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Uni Work\Year 3\FMP\ProcGenTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A42AAE0-5A8B-4DC1-9898-64C2354C6F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8179935-3FD2-4BBF-8D40-E8EA0014CA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{96347398-2AC3-4EB9-A82F-8E2B65190871}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>Bug Tracker</t>
   </si>
@@ -207,6 +207,15 @@
   </si>
   <si>
     <t>Changed EditorGUILayout back to EditorGUI</t>
+  </si>
+  <si>
+    <t>Caves throwing error</t>
+  </si>
+  <si>
+    <t>Cave size being negative</t>
+  </si>
+  <si>
+    <t>Added extra checks to ensure no negative numbers</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1055,9 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -1069,18 +1080,28 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="1"/>
+      <c r="B17" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
+      <c r="I17" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
+      <c r="L17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>

</xml_diff>